<commit_message>
Comment out validation mode sections 06d69a9f962cfb5d3c9a267b717788da570fc830
</commit_message>
<xml_diff>
--- a/nriss-patch-1/ig/CodeSystem-fr-core-cs-mode-validation-identity.xlsx
+++ b/nriss-patch-1/ig/CodeSystem-fr-core-cs-mode-validation-identity.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="75">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-28T15:04:56+00:00</t>
+    <t>2026-09-30T14:05:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -126,7 +126,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>12</t>
+    <t>15</t>
   </si>
   <si>
     <t>Level</t>
@@ -195,7 +195,7 @@
     <t>Extrait d'acte de naissance</t>
   </si>
   <si>
-    <t>LEP</t>
+    <t>LE</t>
   </si>
   <si>
     <t>Livret de famille des parents</t>
@@ -220,6 +220,24 @@
   </si>
   <si>
     <t>Extrait d'acte de naissance, accompagné de la carte Vitale avec photographie</t>
+  </si>
+  <si>
+    <t>IE</t>
+  </si>
+  <si>
+    <t>Identification électronique EIDAS</t>
+  </si>
+  <si>
+    <t>CM</t>
+  </si>
+  <si>
+    <t>Carte militaire</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>Permis de conduire</t>
   </si>
 </sst>
 </file>
@@ -537,7 +555,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -722,6 +740,48 @@
         <v>68</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B14" t="s" s="2">
+        <v>69</v>
+      </c>
+      <c r="C14" t="s" s="2">
+        <v>70</v>
+      </c>
+      <c r="D14" t="s" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B15" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="C15" t="s" s="2">
+        <v>72</v>
+      </c>
+      <c r="D15" t="s" s="2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="C16" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="D16" t="s" s="2">
+        <v>74</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>